<commit_message>
Remove sample rows from inventory workbook
Rows 502-505 in Rings, Bracelets and Necklace were leftover template
examples (price 0, old photo-code format, reusing real article numbers).
Real-workbook test now asserts exact totals per category.
</commit_message>
<xml_diff>
--- a/data/Lunara_Inventory_System_FINAL.xlsx
+++ b/data/Lunara_Inventory_System_FINAL.xlsx
@@ -18035,122 +18035,10 @@
         <v/>
       </c>
     </row>
-    <row r="502" ht="14.25" customHeight="1">
-      <c r="B502" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="C502" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="D502" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E502" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F502" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G502" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="H502" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="I502" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="K502" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="503" ht="14.25" customHeight="1">
-      <c r="B503" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="C503" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="D503" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E503" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F503" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G503" s="1">
-        <v>3.0</v>
-      </c>
-      <c r="H503" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="I503" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="K503" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="504" ht="14.25" customHeight="1">
-      <c r="B504" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="C504" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="D504" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E504" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F504" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G504" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="H504" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="I504" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="K504" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="505" ht="14.25" customHeight="1">
-      <c r="B505" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="C505" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D505" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E505" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F505" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G505" s="1">
-        <v>4.0</v>
-      </c>
-      <c r="H505" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="I505" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="K505" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
+    <row r="502" ht="14.25" customHeight="1"/>
+    <row r="503" ht="14.25" customHeight="1"/>
+    <row r="504" ht="14.25" customHeight="1"/>
+    <row r="505" ht="14.25" customHeight="1"/>
     <row r="506" ht="14.25" customHeight="1"/>
     <row r="507" ht="14.25" customHeight="1"/>
     <row r="508" ht="14.25" customHeight="1"/>
@@ -24718,84 +24606,9 @@
         <v/>
       </c>
     </row>
-    <row r="502" ht="14.25" customHeight="1">
-      <c r="B502" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="C502" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D502" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E502" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F502" s="1">
-        <v>5.0</v>
-      </c>
-      <c r="G502" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="H502" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="J502" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="503" ht="14.25" customHeight="1">
-      <c r="B503" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="C503" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D503" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E503" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F503" s="1">
-        <v>3.0</v>
-      </c>
-      <c r="G503" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="H503" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="J503" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="504" ht="14.25" customHeight="1">
-      <c r="B504" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="C504" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="D504" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E504" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F504" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="G504" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="H504" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="J504" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
+    <row r="502" ht="14.25" customHeight="1"/>
+    <row r="503" ht="14.25" customHeight="1"/>
+    <row r="504" ht="14.25" customHeight="1"/>
     <row r="505" ht="14.25" customHeight="1"/>
     <row r="506" ht="14.25" customHeight="1"/>
     <row r="507" ht="14.25" customHeight="1"/>
@@ -31441,84 +31254,9 @@
         <v/>
       </c>
     </row>
-    <row r="502" ht="14.25" customHeight="1">
-      <c r="B502" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="C502" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="D502" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E502" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F502" s="1">
-        <v>3.0</v>
-      </c>
-      <c r="G502" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="H502" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="J502" s="1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="503" ht="14.25" customHeight="1">
-      <c r="B503" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="C503" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="D503" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E503" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F503" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="G503" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="H503" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="J503" s="1" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="504" ht="14.25" customHeight="1">
-      <c r="B504" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="C504" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="D504" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E504" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F504" s="1">
-        <v>4.0</v>
-      </c>
-      <c r="G504" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="H504" s="1">
-        <v>0.0</v>
-      </c>
-      <c r="J504" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
+    <row r="502" ht="14.25" customHeight="1"/>
+    <row r="503" ht="14.25" customHeight="1"/>
+    <row r="504" ht="14.25" customHeight="1"/>
     <row r="505" ht="14.25" customHeight="1"/>
     <row r="506" ht="14.25" customHeight="1"/>
     <row r="507" ht="14.25" customHeight="1"/>

</xml_diff>